<commit_message>
📊 Horarios actualizados $(date +%Y-%m-%d)
</commit_message>
<xml_diff>
--- a/horarios-141-2026-01-06.xlsx
+++ b/horarios-141-2026-01-06.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,11 +457,16 @@
           <t>Parada</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:59</t>
+          <t>Última actualización: 19:31:13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,11 +487,12 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ejecuciones: 18 filas</t>
+          <t>Ejecuciones: 35 filas únicas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -507,6 +513,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -532,6 +539,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -557,6 +565,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -582,6 +591,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -607,6 +617,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -632,6 +643,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -657,6 +669,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -682,6 +695,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -707,6 +721,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -732,6 +747,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -757,6 +773,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -782,6 +799,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -807,6 +825,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -832,6 +851,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -857,6 +877,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -882,6 +903,7 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -905,6 +927,449 @@
       <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>9</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>19</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>21</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>29</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>39</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>40</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20:13</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>42</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>53</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>82</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>85</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>86</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>94</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>97</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
         </is>
       </c>
     </row>
@@ -919,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -948,11 +1413,16 @@
           <t>Parada</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:59</t>
+          <t>Última actualización: 19:31:13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -973,11 +1443,12 @@
           <t>LP1912</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ejecuciones: 2 filas</t>
+          <t>Ejecuciones: 5 filas únicas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -996,6 +1467,85 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>53</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>97</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>19:31:02</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1039,11 +1589,16 @@
           <t>Parada</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Última actualización: 19:10:59</t>
+          <t>Última actualización: 19:31:13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1064,11 +1619,12 @@
           <t>L6203</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Ejecuciones: 2 filas</t>
+          <t>Ejecuciones: 3 filas únicas</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1087,6 +1643,33 @@
       <c r="E3" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>23</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>19:31:08</t>
         </is>
       </c>
     </row>

</xml_diff>